<commit_message>
modified:   .gitignore 	modified:   pity.xlsx 	deleted:    ~$pity.xlsx
</commit_message>
<xml_diff>
--- a/pity.xlsx
+++ b/pity.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Code\Algorithm\Gacha\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9879BEBE-813B-42EF-8822-69634B73FAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="3443" yWindow="1943" windowWidth="17280" windowHeight="11587" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,26 +24,206 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>p(k)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>description</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>k=0…72</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>p=0.6%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>k=73…88</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>p = 0.006 + 0.06·(k-72)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>k=89</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>p=100%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>基础出货率</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>软保底线性提升，第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>74</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>抽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DengXian"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>≈</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 6.6%</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>保底</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="等线"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="DengXian"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="1"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -45,12 +231,183 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF8EA9C1"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EA9C1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF8EA9C1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF8EA9C1"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EA9C1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF8EA9C1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EA9C1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF8EA9C1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF8EA9C1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EA9C1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF8EA9C1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF8EA9C1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF8EA9C1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EA9C1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF8EA9C1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF8EA9C1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EA9C1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF8EA9C1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF8EA9C1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF8EA9C1"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF8EA9C1"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF8EA9C1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF8EA9C1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF8EA9C1"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -329,11 +686,85 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="700" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{72B2986C-28AE-4803-A9F1-D8D9B726B99C}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;1b33ddac-79aa-4965-9f04-2e3aad7388d7&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="13.9"/>
+  <cols>
+    <col min="1" max="1" width="14.73046875" customWidth="1"/>
+    <col min="2" max="2" width="22.3984375" customWidth="1"/>
+    <col min="3" max="3" width="30.06640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="14.25" thickBot="1"/>
+    <row r="2" spans="1:3" ht="28.05" customHeight="1">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="24" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="24" customHeight="1">
+      <c r="A4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="24" customHeight="1" thickBot="1">
+      <c r="A5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>